<commit_message>
Add concepts of Evaluation and selection of models
</commit_message>
<xml_diff>
--- a/docs/teoria/tablas/ejercicio_13_aprendizaje_automatico.xlsx
+++ b/docs/teoria/tablas/ejercicio_13_aprendizaje_automatico.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juana\ETSII_IA\docs\teoria\tablas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C1C5E152-54D9-4422-987C-E2E2C50C1B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B589F19F-957A-40E1-9CDE-B68829B75A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{0E25C846-6A45-4F7C-8946-341996EB7490}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{0E25C846-6A45-4F7C-8946-341996EB7490}"/>
   </bookViews>
   <sheets>
-    <sheet name="ejercicio_13_aprendizaje_automa" sheetId="1" r:id="rId1"/>
+    <sheet name="kNN_ejercicio_13" sheetId="1" r:id="rId1"/>
+    <sheet name="kNN_ejercicio_16" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
   <si>
     <t>Aluminio</t>
   </si>
@@ -132,6 +133,21 @@
   </si>
   <si>
     <t>Euclidea_E3</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Anchura máxima </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Altura basio-bregmática </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Longitud basioloalveolar </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Altura nasal </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Época </t>
   </si>
 </sst>
 </file>
@@ -141,7 +157,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,6 +295,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -625,7 +649,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -635,6 +659,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2003,4 +2028,139 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F28A81-73F5-40D1-B9C1-8AF16FAECDF5}">
+  <dimension ref="B2:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>131</v>
+      </c>
+      <c r="C3">
+        <v>138</v>
+      </c>
+      <c r="D3">
+        <v>89</v>
+      </c>
+      <c r="E3">
+        <v>49</v>
+      </c>
+      <c r="F3">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>125</v>
+      </c>
+      <c r="C4">
+        <v>131</v>
+      </c>
+      <c r="D4">
+        <v>92</v>
+      </c>
+      <c r="E4">
+        <v>48</v>
+      </c>
+      <c r="F4">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <v>131</v>
+      </c>
+      <c r="C5">
+        <v>132</v>
+      </c>
+      <c r="D5">
+        <v>99</v>
+      </c>
+      <c r="E5">
+        <v>50</v>
+      </c>
+      <c r="F5">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <v>124</v>
+      </c>
+      <c r="C6">
+        <v>138</v>
+      </c>
+      <c r="D6">
+        <v>101</v>
+      </c>
+      <c r="E6">
+        <v>48</v>
+      </c>
+      <c r="F6">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>133</v>
+      </c>
+      <c r="C7">
+        <v>134</v>
+      </c>
+      <c r="D7">
+        <v>97</v>
+      </c>
+      <c r="E7">
+        <v>48</v>
+      </c>
+      <c r="F7">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" s="5">
+        <v>138</v>
+      </c>
+      <c r="C8" s="5">
+        <v>134</v>
+      </c>
+      <c r="D8" s="5">
+        <v>98</v>
+      </c>
+      <c r="E8" s="5">
+        <v>45</v>
+      </c>
+      <c r="F8" s="5">
+        <v>3300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>